<commit_message>
Auto-discover new transfer links daily; refresh World Cup stats to matchday 2
</commit_message>
<xml_diff>
--- a/data/liverpool_data.xlsx
+++ b/data/liverpool_data.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="News (ranked)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Source credibility" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Squad" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Transfers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Injuries" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News (ranked)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source credibility" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Squad" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Injuries" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'News (ranked)'!$A$1:$H$31</definedName>
@@ -530,31 +530,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>‘When you look at him…’ – Carragher gives Diomande transfer verdict amid comparison to LFC legends</t>
+          <t>The Transfer DealSheet: Latest on Man Utd, Arsenal, Liverpool, Real Madrid and more - The Athletic - The New York Times</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Empire of the Kop</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G3" t="n">
-        <v>85.09999999999999</v>
+        <v>85</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.empireofthekop.com/2026/06/22/carragher-gives-diomande-transfer-verdict-amid-salah-mane-comparisons/</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQNFlIVzZic2NnVHc2Yjl3SFpQRE1UZjhOYm02NU5aU2pkSlNpYUJkSkpxZFU4bGtoLWZrNXV2TmZYSGF5bHpENjlFaG1Uejh6NHUxOXUtOGZkUXU5ZWVyMHhYLUNXSXBtcDZETkFtdlVLSkNuZGNjZFdsbWRLMmE3LWUwUXlLVjBmUGxMc0EzWG9id19VS3FtRmZjay1rZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -569,12 +569,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>The Transfer DealSheet: Latest on Man Utd, Arsenal, Liverpool, Real Madrid and more - The Athletic - The New York Times</t>
+          <t>Liverpool 'have an agreement' with Yan Diomande and ONE step away from record-breaking deal – report - Liverpool FC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>Liverpool FC</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -588,7 +588,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxQNFlIVzZic2NnVHc2Yjl3SFpQRE1UZjhOYm02NU5aU2pkSlNpYUJkSkpxZFU4bGtoLWZrNXV2TmZYSGF5bHpENjlFaG1Uejh6NHUxOXUtOGZkUXU5ZWVyMHhYLUNXSXBtcDZETkFtdlVLSkNuZGNjZFdsbWRLMmE3LWUwUXlLVjBmUGxMc0EzWG9id19VS3FtRmZjay1rZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNNkpzNkRPLXBvenVnQlBUZlFKOEY1aHRkYmdjOUZRTGFnaXhzNmdNR3IwOEIxTGZOc1g4QlVhN05PMDMxNjZXQm9zMGJObkZJRlljQ1RRTXR3YTRrQm5KX2FNOE5zX3JjOFVWVFdQN09GWFdZNFhNbGpGc1dESU5kM2t0eXFZeGtBcnlFODJQUFVVRmp1cVVqVHM5UmdTa09DeGNqVGMyTWIydmdYX0FkeXhkQmp0X3PSAb8BQVVfeXFMT0tjZXhCSXktell1ZGhXRi1QWGJoZXpJenVaUTcxQU9IdWF0QWpmSXM3T3d5bUhqR21TX0lkdkFuN1JQQ2VxejI0aHNZTVA1WlRCSjUzclZYbUVfNml5YV9Zc01EUnJOQ0lwMk5ucXpBNDdPcXhkNVVMdXlGbjZOcGktT1hTMEpMUlpFeW9SYUxEb2l0X2ZTUENxRlZzc0kwZUZOcHFqaGNUV2stRWdfamFUamlxbHBjeG9mUzBDN00?oc=5</t>
         </is>
       </c>
     </row>
@@ -603,12 +603,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Liverpool 'have an agreement' with Yan Diomande and ONE step away from record-breaking deal – report - Liverpool FC</t>
+          <t>Liverpool Cody Gakpo World Cup Form Interests Tottenham Hotspur - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Liverpool FC</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -622,7 +622,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitwFBVV95cUxNNkpzNkRPLXBvenVnQlBUZlFKOEY1aHRkYmdjOUZRTGFnaXhzNmdNR3IwOEIxTGZOc1g4QlVhN05PMDMxNjZXQm9zMGJObkZJRlljQ1RRTXR3YTRrQm5KX2FNOE5zX3JjOFVWVFdQN09GWFdZNFhNbGpGc1dESU5kM2t0eXFZeGtBcnlFODJQUFVVRmp1cVVqVHM5UmdTa09DeGNqVGMyTWIydmdYX0FkeXhkQmp0X3PSAb8BQVVfeXFMT0tjZXhCSXktell1ZGhXRi1QWGJoZXpJenVaUTcxQU9IdWF0QWpmSXM3T3d5bUhqR21TX0lkdkFuN1JQQ2VxejI0aHNZTVA1WlRCSjUzclZYbUVfNml5YV9Zc01EUnJOQ0lwMk5ucXpBNDdPcXhkNVVMdXlGbjZOcGktT1hTMEpMUlpFeW9SYUxEb2l0X2ZTUENxRlZzc0kwZUZOcHFqaGNUV2stRWdfamFUamlxbHBjeG9mUzBDN00?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbFRRWHR5VFJWeXJmUmd6Uk5hbXl0T3VHUGVaMWFqU3EyTkFFejdxdHhYU1hfZm0zNVVCVlEySDh1MzFsWlluWWhuR1VYRWhyR0JVVldvcGZyOXVLYXNHdDdKcEw2d3ljTlptTDNUa1ZHTmpNMnBCZ2s4ZXpGdE5DdGtWcWJsbmFya1gtVERzR2lLZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -632,12 +632,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Liverpool Cody Gakpo World Cup Form Interests Tottenham Hotspur - readliverpoolfc.com</t>
+          <t>Virgil van Dijk Sets Netherlands World Cup Target As Liverpool Watch On - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikgFBVV95cUxQbFRRWHR5VFJWeXJmUmd6Uk5hbXl0T3VHUGVaMWFqU3EyTkFFejdxdHhYU1hfZm0zNVVCVlEySDh1MzFsWlluWWhuR1VYRWhyR0JVVldvcGZyOXVLYXNHdDdKcEw2d3ljTlptTDNUa1ZHTmpNMnBCZ2s4ZXpGdE5DdGtWcWJsbmFya1gtVERzR2lLZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNVG45VEtUeVpKdXBidm5xMVFvWXZ1Tjg2cUhiTjJfb0ZDR0k4VDRwWTVBNExyUTJpRVpsYVRIeDB5U1FHczkwNHk1TlBHNmlVMFk3OTBwb3hlS1lVWmZTZVRKUFNOdzV1dE5zSXg1VDFxaGw3WVd1OHFPZjNvTVllZWlvclozM1R2SExOMXFSMFZiNmlkUU1mbA?oc=5</t>
         </is>
       </c>
     </row>
@@ -666,31 +666,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Virgil van Dijk Sets Netherlands World Cup Target As Liverpool Watch On - readliverpoolfc.com</t>
+          <t>How can Liverpool get the best out of World Cup versions of Cody Gakpo and Alexander Isak? - The New York Times</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>readliverpoolfc.com</t>
+          <t>The New York Times</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G7" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNVG45VEtUeVpKdXBidm5xMVFvWXZ1Tjg2cUhiTjJfb0ZDR0k4VDRwWTVBNExyUTJpRVpsYVRIeDB5U1FHczkwNHk1TlBHNmlVMFk3OTBwb3hlS1lVWmZTZVRKUFNOdzV1dE5zSXg1VDFxaGw3WVd1OHFPZjNvTVllZWlvclozM1R2SExOMXFSMFZiNmlkUU1mbA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNZTN3V3BCeTlGMDdxWDBSblRhTjNzRnFpVC1Zc2RoaDNUbWpqR0FqclVxcC0zWk9Iem5qXzZQSThZWW8zQlhqOXZSUk9uVGhmZjl5aDNxb295eDNldWduWk8zLUcwbXExc1FfMElkSXBzWENuVTlCck95Y2F2TlJyaHNhZy1lUVhDbTF0eDNWT29lb1M3Q2YyUGQ3OWtOc1pqcDB3MDJ3?oc=5</t>
         </is>
       </c>
     </row>
@@ -700,31 +700,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>How can Liverpool get the best out of World Cup versions of Cody Gakpo and Alexander Isak? - The New York Times</t>
+          <t>Report: Andoni Iraola’s stance on Cody Gakpo outlined amid rumours of Liverpool exit</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>Empire of the Kop</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="G8" t="n">
-        <v>82</v>
+        <v>80.3</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxNZTN3V3BCeTlGMDdxWDBSblRhTjNzRnFpVC1Zc2RoaDNUbWpqR0FqclVxcC0zWk9Iem5qXzZQSThZWW8zQlhqOXZSUk9uVGhmZjl5aDNxb295eDNldWduWk8zLUcwbXExc1FfMElkSXBzWENuVTlCck95Y2F2TlJyaHNhZy1lUVhDbTF0eDNWT29lb1M3Q2YyUGQ3OWtOc1pqcDB3MDJ3?oc=5</t>
+          <t>https://www.empireofthekop.com/2026/06/24/iraola-stance-on-gakpo-outlined-amid-rumours-of-liverpool-exit/</t>
         </is>
       </c>
     </row>
@@ -734,17 +734,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Report: Andoni Iraola’s stance on Cody Gakpo outlined amid rumours of Liverpool exit</t>
+          <t>It's coming, Fabrizio Romano confirms Liverpool transfer offer is on the way - Anfield Watch</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Empire of the Kop</t>
+          <t>Anfield Watch</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.empireofthekop.com/2026/06/24/iraola-stance-on-gakpo-outlined-amid-rumours-of-liverpool-exit/</t>
+          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNVG5GYU9YS25oUldLb2pIYnpkNVNPam1VbDMwbk83TWZWNXRRazBNY0tZN0xfTEpuNUZoQW8zZXhWZE1WTVZLU2g4eEFKMmwyU0dWSVFwT2syUHh3OGN3UXo2YlpsMnhnalRBM3VvVEVOMTF2U3lQakZYeTFHLXk5M1EzLXk0THJtOGZnTV9jMk94bzlkV0tLWHQxb0J4Mm54MWNVSE1RdEU2SUEyZUpvVHdZTDVVS1ZHRklvMWpLa25uZw?oc=5</t>
         </is>
       </c>
     </row>
@@ -773,12 +773,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>It's coming, Fabrizio Romano confirms Liverpool transfer offer is on the way - Anfield Watch</t>
+          <t>James Pearce: Liverpool must pay £112m to sign top transfer target - anfieldindex.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Anfield Watch</t>
+          <t>anfieldindex.com</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -792,7 +792,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwgFBVV95cUxNVG5GYU9YS25oUldLb2pIYnpkNVNPam1VbDMwbk83TWZWNXRRazBNY0tZN0xfTEpuNUZoQW8zZXhWZE1WTVZLU2g4eEFKMmwyU0dWSVFwT2syUHh3OGN3UXo2YlpsMnhnalRBM3VvVEVOMTF2U3lQakZYeTFHLXk5M1EzLXk0THJtOGZnTV9jMk94bzlkV0tLWHQxb0J4Mm54MWNVSE1RdEU2SUEyZUpvVHdZTDVVS1ZHRklvMWpLa25uZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQWXg3SDJ3YXFVSVBfNzJUVVJsV2NCc1ZaeGlLZzFSNWZoWmpfaV9xWHhWNUY4VUIza2pyZ3E3eXhsN0puM1FRRUVHMGFDa0dYVEptMURBN01QeWV4eXFqRG5LZG5mTl9KeFp0b3FNd05xbTgwM0drcUUtUFZxa1RtTVZnR2RQOGlqc0t5SEJELXlDZnN2akdNbFdFWU5YejlZTlE?oc=5</t>
         </is>
       </c>
     </row>
@@ -807,26 +807,26 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>James Pearce: Liverpool must pay £112m to sign top transfer target - anfieldindex.com</t>
+          <t>Bradley Barcola issues verdict on Liverpool transfer amid Arsenal 'bid' - Liverpool FC</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>anfieldindex.com</t>
+          <t>Liverpool FC</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G11" t="n">
-        <v>80.3</v>
+        <v>80</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQWXg3SDJ3YXFVSVBfNzJUVVJsV2NCc1ZaeGlLZzFSNWZoWmpfaV9xWHhWNUY4VUIza2pyZ3E3eXhsN0puM1FRRUVHMGFDa0dYVEptMURBN01QeWV4eXFqRG5LZG5mTl9KeFp0b3FNd05xbTgwM0drcUUtUFZxa1RtTVZnR2RQOGlqc0t5SEJELXlDZnN2akdNbFdFWU5YejlZTlE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPdkhxNi1NSzltSk5aVlZzeTBCLUpLeWZ3T09tQ3RYNXN2bWdMNjh0YmEyWTNxOVdnSUdMbDFmQnUtTmlzRk05RmdmZFU1ZlFycTFiaE9fRlhaWVByWG1NZVpGNHJNSjVaUTZSMzFESDZSeHdHcElqajdnWHloUE9ZelNUWHNlbUgwanhJbDlPSGR3MGxIdUZ4SnhiS3g5S0xV0gGoAUFVX3lxTE1QTlFVamkxNXFnUVZrMkVBUXVxSFBXSUNZMjJTR3V6TjVmelZOcncwZnl6MUdfWm9jRTRhWmNWTU5PRkRLUkVhMWlFU05PVXNxR2pzeXdJeDVFU2oxUExkclRPcHRnR1FoMEt4Nm9oekRQbzN0VkFQYk11UnNFc2NFUTNpcHIwLWtuNHZFV3hyU2lxVmVfLXpWNm1zbFF3eGwxTzc2ZWtMOQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bradley Barcola issues verdict on Liverpool transfer amid Arsenal 'bid' - Liverpool FC</t>
+          <t>Liverpool make fresh Bradley Barcola transfer attempt with PSG star 'open to move' - Liverpool FC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMioAFBVV95cUxPdkhxNi1NSzltSk5aVlZzeTBCLUpLeWZ3T09tQ3RYNXN2bWdMNjh0YmEyWTNxOVdnSUdMbDFmQnUtTmlzRk05RmdmZFU1ZlFycTFiaE9fRlhaWVByWG1NZVpGNHJNSjVaUTZSMzFESDZSeHdHcElqajdnWHloUE9ZelNUWHNlbUgwanhJbDlPSGR3MGxIdUZ4SnhiS3g5S0xV0gGoAUFVX3lxTE1QTlFVamkxNXFnUVZrMkVBUXVxSFBXSUNZMjJTR3V6TjVmelZOcncwZnl6MUdfWm9jRTRhWmNWTU5PRkRLUkVhMWlFU05PVXNxR2pzeXdJeDVFU2oxUExkclRPcHRnR1FoMEt4Nm9oekRQbzN0VkFQYk11UnNFc2NFUTNpcHIwLWtuNHZFV3hyU2lxVmVfLXpWNm1zbFF3eGwxTzc2ZWtMOQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPWGNaZDZDVVpGQjFqMXg1TmFhVXE4dUcwbjNCRnVlVWFYZVJLbW1Na0ZGSWs2UHZQMm9CeW92NS1BdG1mY0NyelgyV0IyRHdlSEV1RnAtRmpYVm9ORzktR0FnREdiTmJvSlJKaWpmSUt3X0JLVEg0Z253YWJYUmRnLWxCVjluSVBVbVYtOTZfV3ZjTHZKUnlFM1hUSlJFSklFeFkyNDNPQkvSAbABQVVfeXFMTUQwWUhTSGd3V290UzBTTll1bGJhTXk2TUdSbWd1SEMteFEwajE4YUpRY3ZTa2xZUlRvYjlwM3d3S3dYZjQ4VHBoWkVCTU1jSDQ2SkJtZm1fc1g2d0VhQkZweUxCM0xSLW1zeEtsdGRQQlJuMDZRNnlUQTVOMkwyb1FqckNjbWZEYUlrZTBJaktsc2l6OGh2SFN2UWtzaEZnWmZXSmpHZVFES19hWENMZ3Y?oc=5</t>
         </is>
       </c>
     </row>
@@ -870,17 +870,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Liverpool make fresh Bradley Barcola transfer attempt with PSG star 'open to move' - Liverpool FC</t>
+          <t>Liverpool Transfer News: German Target Felix Nmecha Enquiry Made To Bolster Midfield - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Liverpool FC</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -894,7 +894,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPWGNaZDZDVVpGQjFqMXg1TmFhVXE4dUcwbjNCRnVlVWFYZVJLbW1Na0ZGSWs2UHZQMm9CeW92NS1BdG1mY0NyelgyV0IyRHdlSEV1RnAtRmpYVm9ORzktR0FnREdiTmJvSlJKaWpmSUt3X0JLVEg0Z253YWJYUmRnLWxCVjluSVBVbVYtOTZfV3ZjTHZKUnlFM1hUSlJFSklFeFkyNDNPQkvSAbABQVVfeXFMTUQwWUhTSGd3V290UzBTTll1bGJhTXk2TUdSbWd1SEMteFEwajE4YUpRY3ZTa2xZUlRvYjlwM3d3S3dYZjQ4VHBoWkVCTU1jSDQ2SkJtZm1fc1g2d0VhQkZweUxCM0xSLW1zeEtsdGRQQlJuMDZRNnlUQTVOMkwyb1FqckNjbWZEYUlrZTBJaktsc2l6OGh2SFN2UWtzaEZnWmZXSmpHZVFES19hWENMZ3Y?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOUXVleEpUYlRBWmJxVTNHNS1TQV9YZ2hhVVlSa0lSSXFMeVczUTZyMmJOYmhEWGtLYjFnNV9DWENJZXN1eUFCUGJIdmVUNGpYaklOa3FDU0RkRmxFMEdnZC1fRDdSSmpoejNpRW16SllicVFsOXZONExHTWJzSU5RUGx5Nks?oc=5</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Liverpool Transfer News: German Target Felix Nmecha Enquiry Made To Bolster Midfield - readliverpoolfc.com</t>
+          <t>Alisson Becker Brazil Call Gives Liverpool Early World Cup Watchpoint - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOUXVleEpUYlRBWmJxVTNHNS1TQV9YZ2hhVVlSa0lSSXFMeVczUTZyMmJOYmhEWGtLYjFnNV9DWENJZXN1eUFCUGJIdmVUNGpYaklOa3FDU0RkRmxFMEdnZC1fRDdSSmpoejNpRW16SllicVFsOXZONExHTWJzSU5RUGx5Nks?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOVG1oWVMtajF4RVZyRHJTNjVwbTVNek1uWHUxbVU5bjkzbWVsRVJNa0NOSXNXT0VoTTZDUl9LbS1NVGczVnplaU9WZUsyeF9yWllaeUJSSzlsUTAwSC1QanNlWVA1V3VaTW9oOURISmx5dkZVakFpMUZPcEk4V1NpR21lV0VfZGtRNWc3dFcwQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -1040,31 +1040,31 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Alisson Becker Brazil Call Gives Liverpool Early World Cup Watchpoint - readliverpoolfc.com</t>
+          <t>Eight things you need to know about Liverpool's transfer business this week</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>readliverpoolfc.com</t>
+          <t>Liverpool Echo</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="G18" t="n">
-        <v>80</v>
+        <v>79.3</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOVG1oWVMtajF4RVZyRHJTNjVwbTVNek1uWHUxbVU5bjkzbWVsRVJNa0NOSXNXT0VoTTZDUl9LbS1NVGczVnplaU9WZUsyeF9yWllaeUJSSzlsUTAwSC1QanNlWVA1V3VaTW9oOURISmx5dkZVakFpMUZPcEk4V1NpR21lV0VfZGtRNWc3dFcwQQ?oc=5</t>
+          <t>https://www.liverpoolecho.co.uk/sport/football/transfer-news/eight-things-you-need-know-34173085</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eight things you need to know about Liverpool's transfer business this week</t>
+          <t>Cody Gakpo sent clear Liverpool instruction amid Victor Munoz transfer and Yan Diomande pursuit</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.liverpoolecho.co.uk/sport/football/transfer-news/eight-things-you-need-know-34173085</t>
+          <t>https://www.liverpoolecho.co.uk/sport/football/football-news/cody-gakpo-sent-clear-liverpool-34165667</t>
         </is>
       </c>
     </row>
@@ -1108,31 +1108,31 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cody Gakpo sent clear Liverpool instruction amid Victor Munoz transfer and Yan Diomande pursuit</t>
+          <t>Liverpool target Yan Diomande drops telling transfer hint - 'My agents will sort it' - Liverpool FC</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Liverpool Echo</t>
+          <t>Liverpool FC</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="G20" t="n">
-        <v>79.3</v>
+        <v>77</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.liverpoolecho.co.uk/sport/football/football-news/cody-gakpo-sent-clear-liverpool-34165667</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQYzlNSXBwbEJISnl6R2g0MVFMWmw4emNKN3ppNHJNcnFJeHk1UzA2OXhYTzJHTEFEZEpKcFNuRjJ5TUhoQ2tBNUNuczRjb1Z1Q1FYd0tacktydnJKT2Z5U1BqNnZWUzhsWnFzVnNCLVpJbWo0TzFNeUMwQk9haEVxT1VFNHloSzRGSklPOHZtakJqeUhCZ1YtdzZmbG02eHRQa2M2MWFkZlFCamV1MmJGMmdOTdIBuwFBVV95cUxPSmxyVDdJM202ZWJzSjBLeG9DZWsxMHdaR0xOczdzbW8xX3lPRXhXdFF2NjRyaHIwX3V0cG8zVFk5cHFNQ1JZRGtlU2RnMjBXbWV3ZDNMWjZ0WDlPOC1mZk1iM0QyYXBFZXViZmc1djJfeFd0OWF4OUlvRkV2dXpTSWpqRkJ2RlNlSGNpdzZFTUliZldIYmQ2Z3NER2hDUm1FRjBRaDI3T3VfSlBUNFNvMHFVREEwd2lpd0xV?oc=5</t>
         </is>
       </c>
     </row>
@@ -1142,12 +1142,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Liverpool target Yan Diomande drops telling transfer hint - 'My agents will sort it' - Liverpool FC</t>
+          <t>World Cup: Florian Wirtz features as Germany book place in last 32 - Liverpool FC</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQYzlNSXBwbEJISnl6R2g0MVFMWmw4emNKN3ppNHJNcnFJeHk1UzA2OXhYTzJHTEFEZEpKcFNuRjJ5TUhoQ2tBNUNuczRjb1Z1Q1FYd0tacktydnJKT2Z5U1BqNnZWUzhsWnFzVnNCLVpJbWo0TzFNeUMwQk9haEVxT1VFNHloSzRGSklPOHZtakJqeUhCZ1YtdzZmbG02eHRQa2M2MWFkZlFCamV1MmJGMmdOTdIBuwFBVV95cUxPSmxyVDdJM202ZWJzSjBLeG9DZWsxMHdaR0xOczdzbW8xX3lPRXhXdFF2NjRyaHIwX3V0cG8zVFk5cHFNQ1JZRGtlU2RnMjBXbWV3ZDNMWjZ0WDlPOC1mZk1iM0QyYXBFZXViZmc1djJfeFd0OWF4OUlvRkV2dXpTSWpqRkJ2RlNlSGNpdzZFTUliZldIYmQ2Z3NER2hDUm1FRjBRaDI3T3VfSlBUNFNvMHFVREEwd2lpd0xV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNeVdTY0dsS0dqeEcwaWMycnhXNWo5M0RscDRuT194ckdxUUxEeEJma2swSFdTQUFkSXNzNllGNTVLRWt2QkFtbTlzQkZTWmxoVWpseXZsdnJXdkY3UTVtbThGNXZxVDVMSGduRHpkWnh4REl1NWd0Q3dPcnpES1U2OHR6OTVaWEJ3bHdOUlNaYXhtY3Z0ZWlr0gGfAUFVX3lxTE82aVdzMi1EbFg5RnFrbGV2bmxIVlZjOTZnekJ5bmZLOTFWazZIZzZpb2hyYllDZmdISDJwZVIzVFEyTlRwcWpTTGUwa2swZzByMmtRc0U2dHlRemV6RG5tbkxfMU5oQk1mZWZHTmUyNE5VanNYR0p1LXQ5NmxhTWxWT3kxQ1NUTkEyX3c5Wll2OEotNDlqaUVHbkVUdEVSaw?oc=5</t>
         </is>
       </c>
     </row>
@@ -1176,17 +1176,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>World Cup: Cody Gakpo scores twice as Reds meet in Netherlands v Sweden - Liverpool FC</t>
+          <t>Cody Gakpo Tottenham Interest Confirmed As Liverpool Delay Transfer Decision - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Liverpool FC</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxON1F0dnRxNXlSVjY5ekNXQ0JoVVlvNWlDZDdSNWlEZm1rWTFLbWFxZ0FSSFVpZkViamUway1ucWcteGh2ZFRBTFJqbHI4RUF4UFF3QV8td3V0VXpjN3pIamhJYUw5bGRNUUVtclRrSHdWOERmVlNUdUJsVDZHS0o3eGJOMVhPb09vSEdoT0c4UWhaYzMwQ0JlWGwwOGVsd9IBpgFBVV95cUxNa2VIQzZqQkREWHhrVVhvanI5bEFKbktqV2U0LXR5MFN5dGQwakRxVFdHUlp3UVJGbVlWTWF0NjZrY2tFdGNHZnhUa2ktVzFVTTlQbXNKaV9nZy02M2h4Y01lZi1EYkpURHhaOGY2X0o5Tkh1OU1pdmxoVlFtbUZPYmp5dXlSLV8yQ05oQ0RSTFdLV3hUNEJCV3UzSXVORDJxU0xXYWpn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNRmhFRk90ajR2WmowQUt1SUZGR3BaaXl0d2dmWW1aODV1NzhtakVfdVdYb01RcXZuZUg5T1ljdnhyR0VqeE9QSnkybmVNN1ZBWjlvc2piWWNSWWVRSzVmTVRmdkJTcG9XWmlINzRPNTU1MEhoR1czaC1yUGNjTmliSlkxZHY3OEpBeHljZHNacHhpWjBESkZFXw?oc=5</t>
         </is>
       </c>
     </row>
@@ -1210,31 +1210,31 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>World Cup: Florian Wirtz features as Germany book place in last 32 - Liverpool FC</t>
+          <t>Liverpool sign Víctor Muñoz for £34.5m in first arrival of Andoni Iraola era</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Liverpool FC</t>
+          <t>The Guardian</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G23" t="n">
-        <v>77</v>
+        <v>76.5</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNeVdTY0dsS0dqeEcwaWMycnhXNWo5M0RscDRuT194ckdxUUxEeEJma2swSFdTQUFkSXNzNllGNTVLRWt2QkFtbTlzQkZTWmxoVWpseXZsdnJXdkY3UTVtbThGNXZxVDVMSGduRHpkWnh4REl1NWd0Q3dPcnpES1U2OHR6OTVaWEJ3bHdOUlNaYXhtY3Z0ZWlr0gGfAUFVX3lxTE82aVdzMi1EbFg5RnFrbGV2bmxIVlZjOTZnekJ5bmZLOTFWazZIZzZpb2hyYllDZmdISDJwZVIzVFEyTlRwcWpTTGUwa2swZzByMmtRc0U2dHlRemV6RG5tbkxfMU5oQk1mZWZHTmUyNE5VanNYR0p1LXQ5NmxhTWxWT3kxQ1NUTkEyX3c5Wll2OEotNDlqaUVHbkVUdEVSaw?oc=5</t>
+          <t>https://www.theguardian.com/football/2026/jun/18/victor-munoz-liverpool-newcastle-andoni-iraola-transfer-news</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Cody Gakpo Tottenham Interest Confirmed As Liverpool Delay Transfer Decision - readliverpoolfc.com</t>
+          <t>Liverpool Transfer News: Victor Muñoz signs six-year deal after US medical - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1261,14 +1261,14 @@
         <v>10</v>
       </c>
       <c r="F24" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G24" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNRmhFRk90ajR2WmowQUt1SUZGR3BaaXl0d2dmWW1aODV1NzhtakVfdVdYb01RcXZuZUg5T1ljdnhyR0VqeE9QSnkybmVNN1ZBWjlvc2piWWNSWWVRSzVmTVRmdkJTcG9XWmlINzRPNTU1MEhoR1czaC1yUGNjTmliSlkxZHY3OEpBeHljZHNacHhpWjBESkZFXw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNUGNKZjhPRzZaU3ZiQWpCZF9YTzViRHVTYjlpTDZEWjkzTVZidHRlUjhoNWg5bmNHYjI3Tkp1cHJqSjdZR244YzVpZlYtODhxZ2hFR3lwUC1JZTVKUzhZVjZNSWV0MUpxV3pUcXUwYzhpWDV5cmI2YmlFV3oxNUVLNDh3?oc=5</t>
         </is>
       </c>
     </row>
@@ -1278,31 +1278,31 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Liverpool sign Víctor Muñoz for £34.5m in first arrival of Andoni Iraola era</t>
+          <t>Transfer rumors, news: Tottenham eye move for Liverpool's Gakpo - ESPN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>The Guardian</t>
+          <t>ESPN</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G25" t="n">
-        <v>76.5</v>
+        <v>75.7</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.theguardian.com/football/2026/jun/18/victor-munoz-liverpool-newcastle-andoni-iraola-transfer-news</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPYlo1NGNQeEp5U3hDME1uU0JHN050VjhUZTFPSk1lVk85QjVha2JvY3BqdGo5NE5IU0RaMUE0NTlJbERqaGRPQV9TakQ0UkplQlUzMEdHb01kTjRwVWt2cGotaEdWeWVvSXVzR2YtY3dpZE51SnRObDN4NGFrYmFTZGNjNmNHcm1WQ1l5cDUtTHR0WC1Bd1R2WDM5LXR3YS1QY19BaTBn?oc=5</t>
         </is>
       </c>
     </row>
@@ -1312,31 +1312,31 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Liverpool Transfer News: Victor Muñoz signs six-year deal after US medical - readliverpoolfc.com</t>
+          <t>Fabrizio Romano reveals whether Liverpool will sell Cody Gakpo to Tottenham - Football365</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>readliverpoolfc.com</t>
+          <t>Football365</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F26" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G26" t="n">
-        <v>76</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNUGNKZjhPRzZaU3ZiQWpCZF9YTzViRHVTYjlpTDZEWjkzTVZidHRlUjhoNWg5bmNHYjI3Tkp1cHJqSjdZR244YzVpZlYtODhxZ2hFR3lwUC1JZTVKUzhZVjZNSWV0MUpxV3pUcXUwYzhpWDV5cmI2YmlFV3oxNUVLNDh3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX2J6X01KNm0yYVFHWHNSMmdNRTc0Yk9zaVpyTmIycjByVGIxOXYxSy12Q0xEZWU1dHY1cVYyUjB4cTZRd2pwMVcwU2JoV1l1OWNjd0xDalhqbDYzb1lybVA5Qmc3UUNTcmpuN1QwbFNOLWJ1c0JqS1RkU2pZbWU1MHZhc3hOV0VBSUpjdEdkaHdYdGE3bGFYZmJR?oc=5</t>
         </is>
       </c>
     </row>
@@ -1351,26 +1351,26 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Transfer rumors, news: Tottenham eye move for Liverpool's Gakpo - ESPN</t>
+          <t>Superb £86m Liverpool swoop boosted by Fabrizio Romano as rival deal collapses - MSN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ESPN</t>
+          <t>MSN</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F27" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G27" t="n">
-        <v>75.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPYlo1NGNQeEp5U3hDME1uU0JHN050VjhUZTFPSk1lVk85QjVha2JvY3BqdGo5NE5IU0RaMUE0NTlJbERqaGRPQV9TakQ0UkplQlUzMEdHb01kTjRwVWt2cGotaEdWeWVvSXVzR2YtY3dpZE51SnRObDN4NGFrYmFTZGNjNmNHcm1WQ1l5cDUtTHR0WC1Bd1R2WDM5LXR3YS1QY19BaTBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOV2JMc09SY1dLRC01Uks2UW84ZHNlQThGSFp0d3FLZ190SGQ3TWRMUzNHcEdGYnBQYmFtNjgwWkw4SWozN3dfZmVuRHQ1RnVxZVNkRXpvX0xHZUdXLWpHWHlSQW1yeHNKc2VKSkNBc3g0Y2pDZXlwcHNQNWE1LXBLb1FjZWhSSlFoaWQ1QlhWWHdZd21BYVV3SUF5N2JPZ2lJdlhleHBJNW9BM2t3eGU4WHJOSV9SWUROSTRSWXZwQzBaRGxLWUE?oc=5</t>
         </is>
       </c>
     </row>
@@ -1385,12 +1385,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fabrizio Romano reveals whether Liverpool will sell Cody Gakpo to Tottenham - Football365</t>
+          <t>Liverpool rocked as Arsenal 'pushing' to complete £60m signing 'now' – Fabrizio Romano - MSN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Football365</t>
+          <t>MSN</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX2J6X01KNm0yYVFHWHNSMmdNRTc0Yk9zaVpyTmIycjByVGIxOXYxSy12Q0xEZWU1dHY1cVYyUjB4cTZRd2pwMVcwU2JoV1l1OWNjd0xDalhqbDYzb1lybVA5Qmc3UUNTcmpuN1QwbFNOLWJ1c0JqS1RkU2pZbWU1MHZhc3hOV0VBSUpjdEdkaHdYdGE3bGFYZmJR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiowNBVV95cUxPcEZOa0hxYnNKMmVhUVk5UzYwSWtMcmJidjRibGJueHJubXhuVUs3WVZpR2NfVmZ2b0FJZU0tbmxGYzZlc3ZvSk81RWdnYU1nQ2VyM0ctbm1UOVhrRmp3SlBucVIwMEk5QklMcEFFdEZaYWRWaVdDRHZqLWJXb2t6MHVrdFJYamJpbjhWYnVnX0taYmJOZVpPNmZySlJKZEc2OWRLU0FJc2ZtWU9zd3FFdnB3VUN6b1lVeG9ZYlh1U2lDdGxwUEw5TTVHUVMwVVpFX05VZ0JSbUN1X01lSjE1d3hMR2dvemZlZ25wQXJEd0l2R081SUVfRndKSjlHajRaZUZTMG00RXloemIyT015ak5DN2lxY0pJSVhqeXV6UHBxeE9pa1NweTB0OXg3eXJ3MUdwZDZ3cVk2MnpCNC13ZmJ4cEhIWnB4cnJrVGFnTDR3NHhqZUk0T3BIMlNHRFlXMHY0OG9hbmNVTnhqVGUtS2RmOXlEVlByQWhnajNnQ1lWZVA5V2dDd2tBWDY2aGdOY2hkODBaUkUxaVBqZERvMVhNWQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Superb £86m Liverpool swoop boosted by Fabrizio Romano as rival deal collapses - MSN</t>
+          <t>Fabrizio Romano confirms Liverpool missed out on perfect Conor Bradley replacement - Anfield Watch</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>Anfield Watch</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOV2JMc09SY1dLRC01Uks2UW84ZHNlQThGSFp0d3FLZ190SGQ3TWRMUzNHcEdGYnBQYmFtNjgwWkw4SWozN3dfZmVuRHQ1RnVxZVNkRXpvX0xHZUdXLWpHWHlSQW1yeHNKc2VKSkNBc3g0Y2pDZXlwcHNQNWE1LXBLb1FjZWhSSlFoaWQ1QlhWWHdZd21BYVV3SUF5N2JPZ2lJdlhleHBJNW9BM2t3eGU4WHJOSV9SWUROSTRSWXZwQzBaRGxLWUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOVWtUSjlBeHRjaHh0QmREMHpEU05EaEhQZnpwNVFqRGkyWVdNVUpCUE5tNEJKcFoyRzhhMUtFZE5NSkp6MG5aY0ZzaVVPMWpkRHNjbmFEckFRUENYZGViSno5ckxTbmVMcGFiSE14N1ZwcTBFVUpJLXI4VjV5Z2tRVnZBTklja1ZsaGVBbGxSNFdwdzMtQzEzazBMTDMxZlJwTVZiclZSVHV0UUszUHNFbVI2MGJ2eWVwU19CVEdGN3Bqa1ZQWXpIaUhkak4?oc=5</t>
         </is>
       </c>
     </row>
@@ -1448,17 +1448,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>‘For sure…’ – Fabrizio Romano confirms Premier League interest in confident Liverpool star - MSN</t>
+          <t>Fabrizio Romano confirms Liverpool talks for sensational midfielder - Anfield Watch</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>Anfield Watch</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi1AFBVV95cUxOMVRBQmFCOTl0VFpXbWF1aVpqdk1ESnZIMG5ZMVNWS29EbUE2Z09zMjdzOUIzZ1BZN3lXQkxocXJ1cnNkYzdFYlpUbHJMOXA4OWpkcFRiUlpaeHVGWkVBMnNCcmQ1X042eGtMT2dka3dnY1VDRmhVZ0JuRlhYTmVmc3RsTmRHNEg2YzZhVXBBWVc2SDBfcHRUaVRnWUVmVWxnYjJSYURYcG4zR1A1TDFLRXVpSmhaODF3ZEJmQjlDYnRrT2NkSzlSS21wYUkycXZpckpJTw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPdVRCMW5CSVlJc2pwei1ZY044dVktUzczWEdpbUVNcm8yU0FpWU9lUTJIUkdTX29BSUYzY1hkeFJGaHF2R0x5NHI1b0RDWTF2WkttUk8xdkVWWTdCVl9PZm9tVEZJcmFraTRBaDc2Y0tXS1pwUUlZa0pYQl9wU2dWbDFKdjE3TExPVkVNaFFkSXUyNmhIT3loY1pDNDlESFRMMzliX1BDckJGanpUUWFuM0QxUHRDSVNz?oc=5</t>
         </is>
       </c>
     </row>
@@ -1482,17 +1482,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Liverpool rocked as Arsenal 'pushing' to complete £60m signing 'now' – Fabrizio Romano - MSN</t>
+          <t>Ornstein Drops €100M BOMBA! Liverpool’s Diomande Move REJECTED Jake Gyllenhaal (jKheLn24tz) - Fathom Journal</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>Fathom Journal</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowNBVV95cUxPcEZOa0hxYnNKMmVhUVk5UzYwSWtMcmJidjRibGJueHJubXhuVUs3WVZpR2NfVmZ2b0FJZU0tbmxGYzZlc3ZvSk81RWdnYU1nQ2VyM0ctbm1UOVhrRmp3SlBucVIwMEk5QklMcEFFdEZaYWRWaVdDRHZqLWJXb2t6MHVrdFJYamJpbjhWYnVnX0taYmJOZVpPNmZySlJKZEc2OWRLU0FJc2ZtWU9zd3FFdnB3VUN6b1lVeG9ZYlh1U2lDdGxwUEw5TTVHUVMwVVpFX05VZ0JSbUN1X01lSjE1d3hMR2dvemZlZ25wQXJEd0l2R081SUVfRndKSjlHajRaZUZTMG00RXloemIyT015ak5DN2lxY0pJSVhqeXV6UHBxeE9pa1NweTB0OXg3eXJ3MUdwZDZ3cVk2MnpCNC13ZmJ4cEhIWnB4cnJrVGFnTDR3NHhqZUk0T3BIMlNHRFlXMHY0OG9hbmNVTnhqVGUtS2RmOXlEVlByQWhnajNnQ1lWZVA5V2dDd2tBWDY2aGdOY2hkODBaUkUxaVBqZERvMVhNWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1qQXI1OWcyNmNaeW5GekhZUlBCTGNHVU1nQnZZbWctV1BUNnlGdHRmdU9CNFlHa3JWNEpGb2tUNmo4ZGtIVkJ4RURkLXZqNjBPX1ZWd3h3T0RHMHF2c2pacnhIYmw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stricter auto-discovery: only surface a player linked to LFC in 3+ reports across 2+ outlets
</commit_message>
<xml_diff>
--- a/data/liverpool_data.xlsx
+++ b/data/liverpool_data.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="News (ranked)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Source credibility" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Squad" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Transfers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Injuries" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="News (ranked)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source credibility" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Squad" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Injuries" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'News (ranked)'!$A$1:$H$31</definedName>
@@ -632,31 +632,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Liverpool transfer news, rumours and gossip: Live updates and latest on deals, signings, loans and contracts - Sky Sports</t>
+          <t>Virgil van Dijk Sets Netherlands World Cup Target As Liverpool Watch On - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sky Sports</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G6" t="n">
-        <v>82.2</v>
+        <v>85</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi8AFBVV95cUxOS2lFTGpEa2w5NVVFcjNpZVB4SDlMTFVwVjY1MUk5Q1Bza2hEeUl2V1Q0dGNfaGxuc1VCZHdNNk5pSmFJZzFkbWV0MnZxd09yUkpFYUNQNFRYOTRzaXdBcDF2S1Q0RTMxemhCSnBWX1lBWHY4OVNuaUhKWThqVTQ3MGI4U0ZhZ3BfYnlIVG0yYVJFbU1CUlZLdnRZU1R4aUR1WG5VT1V2RXZpTExvMHNFcml4UmRWQ205VnNzb2UzdUtXRURET1VsZzgxY2ZUQXdueGJGTG1WU0tTOXJHamdWT1pwajRWTDdMS1RFcW0tMmU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNVG45VEtUeVpKdXBidm5xMVFvWXZ1Tjg2cUhiTjJfb0ZDR0k4VDRwWTVBNExyUTJpRVpsYVRIeDB5U1FHczkwNHk1TlBHNmlVMFk3OTBwb3hlS1lVWmZTZVRKUFNOdzV1dE5zSXg1VDFxaGw3WVd1OHFPZjNvTVllZWlvclozM1R2SExOMXFSMFZiNmlkUU1mbA?oc=5</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Liverpool Victor Muñoz Give Liverpool World Cup Wait After Spain Win - readliverpoolfc.com</t>
+          <t>Liverpool Transfer News: German Target Felix Nmecha Enquiry Made To Bolster Midfield - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPUFV5VUprWlZSRkpJRVRYQl9NSy1uaU4xRG1ialhXMnNTRk5KWjBBN1p5RUN3YUxqNENndGlZc2V6N1hKTG9oRVFOTXJCaVc3M3YtRWVLdHZkZWJzenVaUEJYWVBHd3hIRXRsODhGdlMxNlZhSTBxa1VSdy14QldkTTFpMWNCVkl0TnBuUGs5ajVsZllsYkE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOUXVleEpUYlRBWmJxVTNHNS1TQV9YZ2hhVVlSa0lSSXFMeVczUTZyMmJOYmhEWGtLYjFnNV9DWENJZXN1eUFCUGJIdmVUNGpYaklOa3FDU0RkRmxFMEdnZC1fRDdSSmpoejNpRW16SllicVFsOXZONExHTWJzSU5RUGx5Nks?oc=5</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cody Gakpo Competition Grows As Liverpool Add Victor Munoz - readliverpoolfc.com</t>
+          <t>Andoni Iraola Liverpool Opener At Newcastle Confirmed Ahead Of 2026/27 Season - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRWlFdDRnOVgxOGtEM2twMEtZUWlEak9QaG4yN2FYSFZqQ0Q0UVExTmxRYW9RMW91LU90TC0wSUVRYWZua0FVS3JGNlppMGVZQU94UG5YMGpVandKMWtkU2lhMGlOQVdMNG4xbEZ2NXR6R3gwNVdKd0d6cklDWEc2NmEzUzJvTWhmN1hHRA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiigFBVV95cUxNZlhTUGF6SkhNUjl5d1lUMXZaS3d2eURMbThxVHZnS01haTdqT2ROSk9Ca2hFSUtTWEFDT25icURFUl9IYnowX3dsY0h6WEtMajRWeEpxNGQzTGktU011aE5KLXpFQ3lZaUhydERucUtfNkpKSlc2SU5KUDFlU29icXNiT0RGWE9neVE?oc=5</t>
         </is>
       </c>
     </row>
@@ -938,12 +938,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Alisson Becker Brazil Call Gives Liverpool Early World Cup Watchpoint - readliverpoolfc.com</t>
+          <t>Liverpool Victor Muñoz Give Liverpool World Cup Wait After Spain Win - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOVG1oWVMtajF4RVZyRHJTNjVwbTVNek1uWHUxbVU5bjkzbWVsRVJNa0NOSXNXT0VoTTZDUl9LbS1NVGczVnplaU9WZUsyeF9yWllaeUJSSzlsUTAwSC1QanNlWVA1V3VaTW9oOURISmx5dkZVakFpMUZPcEk4V1NpR21lV0VfZGtRNWc3dFcwQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxPUFV5VUprWlZSRkpJRVRYQl9NSy1uaU4xRG1ialhXMnNTRk5KWjBBN1p5RUN3YUxqNENndGlZc2V6N1hKTG9oRVFOTXJCaVc3M3YtRWVLdHZkZWJzenVaUEJYWVBHd3hIRXRsODhGdlMxNlZhSTBxa1VSdy14QldkTTFpMWNCVkl0TnBuUGs5ajVsZllsYkE?oc=5</t>
         </is>
       </c>
     </row>
@@ -972,31 +972,31 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eight things you need to know about Liverpool's transfer business this week</t>
+          <t>Cody Gakpo Competition Grows As Liverpool Add Victor Munoz - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Liverpool Echo</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G16" t="n">
-        <v>79.3</v>
+        <v>80</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.liverpoolecho.co.uk/sport/football/transfer-news/eight-things-you-need-know-34173085</t>
+          <t>https://news.google.com/rss/articles/CBMijAFBVV95cUxQRWlFdDRnOVgxOGtEM2twMEtZUWlEak9QaG4yN2FYSFZqQ0Q0UVExTmxRYW9RMW91LU90TC0wSUVRYWZua0FVS3JGNlppMGVZQU94UG5YMGpVandKMWtkU2lhMGlOQVdMNG4xbEZ2NXR6R3gwNVdKd0d6cklDWEc2NmEzUzJvTWhmN1hHRA?oc=5</t>
         </is>
       </c>
     </row>
@@ -1006,31 +1006,31 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cody Gakpo sent clear Liverpool instruction amid Victor Munoz transfer and Yan Diomande pursuit</t>
+          <t>Alisson Becker Brazil Call Gives Liverpool Early World Cup Watchpoint - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Liverpool Echo</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G17" t="n">
-        <v>79.3</v>
+        <v>80</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.liverpoolecho.co.uk/sport/football/football-news/cody-gakpo-sent-clear-liverpool-34165667</t>
+          <t>https://news.google.com/rss/articles/CBMijwFBVV95cUxOVG1oWVMtajF4RVZyRHJTNjVwbTVNek1uWHUxbVU5bjkzbWVsRVJNa0NOSXNXT0VoTTZDUl9LbS1NVGczVnplaU9WZUsyeF9yWllaeUJSSzlsUTAwSC1QanNlWVA1V3VaTW9oOURISmx5dkZVakFpMUZPcEk4V1NpR21lV0VfZGtRNWc3dFcwQQ?oc=5</t>
         </is>
       </c>
     </row>
@@ -1040,31 +1040,31 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Liverpool target Yan Diomande drops telling transfer hint - 'My agents will sort it' - Liverpool FC</t>
+          <t>Eight things you need to know about Liverpool's transfer business this week</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Liverpool FC</t>
+          <t>Liverpool Echo</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G18" t="n">
-        <v>77</v>
+        <v>79.3</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQYzlNSXBwbEJISnl6R2g0MVFMWmw4emNKN3ppNHJNcnFJeHk1UzA2OXhYTzJHTEFEZEpKcFNuRjJ5TUhoQ2tBNUNuczRjb1Z1Q1FYd0tacktydnJKT2Z5U1BqNnZWUzhsWnFzVnNCLVpJbWo0TzFNeUMwQk9haEVxT1VFNHloSzRGSklPOHZtakJqeUhCZ1YtdzZmbG02eHRQa2M2MWFkZlFCamV1MmJGMmdOTdIBuwFBVV95cUxPSmxyVDdJM202ZWJzSjBLeG9DZWsxMHdaR0xOczdzbW8xX3lPRXhXdFF2NjRyaHIwX3V0cG8zVFk5cHFNQ1JZRGtlU2RnMjBXbWV3ZDNMWjZ0WDlPOC1mZk1iM0QyYXBFZXViZmc1djJfeFd0OWF4OUlvRkV2dXpTSWpqRkJ2RlNlSGNpdzZFTUliZldIYmQ2Z3NER2hDUm1FRjBRaDI3T3VfSlBUNFNvMHFVREEwd2lpd0xV?oc=5</t>
+          <t>https://www.liverpoolecho.co.uk/sport/football/transfer-news/eight-things-you-need-know-34173085</t>
         </is>
       </c>
     </row>
@@ -1074,31 +1074,31 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cody Gakpo Tottenham Interest Confirmed As Liverpool Delay Transfer Decision - readliverpoolfc.com</t>
+          <t>Cody Gakpo sent clear Liverpool instruction amid Victor Munoz transfer and Yan Diomande pursuit</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>readliverpoolfc.com</t>
+          <t>Liverpool Echo</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F19" t="n">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="G19" t="n">
-        <v>77</v>
+        <v>79.3</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNRmhFRk90ajR2WmowQUt1SUZGR3BaaXl0d2dmWW1aODV1NzhtakVfdVdYb01RcXZuZUg5T1ljdnhyR0VqeE9QSnkybmVNN1ZBWjlvc2piWWNSWWVRSzVmTVRmdkJTcG9XWmlINzRPNTU1MEhoR1czaC1yUGNjTmliSlkxZHY3OEpBeHljZHNacHhpWjBESkZFXw?oc=5</t>
+          <t>https://www.liverpoolecho.co.uk/sport/football/football-news/cody-gakpo-sent-clear-liverpool-34165667</t>
         </is>
       </c>
     </row>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ivory Coast beats Ecuador at World Cup as Liverpool target Yan Diomande goes global - The Athletic - The New York Times</t>
+          <t>Liverpool target Yan Diomande drops telling transfer hint - 'My agents will sort it' - Liverpool FC</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>The New York Times</t>
+          <t>Liverpool FC</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxPdWN4Y0FxNVVWckhtYXVmSEpfUUxVR2hZLXUzcXNJc3Y1OHM3U2hxT0tBSlcwZGszZU9iU0RzWl9hQlhsOGFRNlB6Ym1CTU0wcnlaLTduNWtHTi0wNlBQOW5HejJaRVl2aFdOdkhuWmpIQ1QwbV9UUTMzdWZBZ0V2Snp1WDRrMElxTWk4Z0l4azU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQYzlNSXBwbEJISnl6R2g0MVFMWmw4emNKN3ppNHJNcnFJeHk1UzA2OXhYTzJHTEFEZEpKcFNuRjJ5TUhoQ2tBNUNuczRjb1Z1Q1FYd0tacktydnJKT2Z5U1BqNnZWUzhsWnFzVnNCLVpJbWo0TzFNeUMwQk9haEVxT1VFNHloSzRGSklPOHZtakJqeUhCZ1YtdzZmbG02eHRQa2M2MWFkZlFCamV1MmJGMmdOTdIBuwFBVV95cUxPSmxyVDdJM202ZWJzSjBLeG9DZWsxMHdaR0xOczdzbW8xX3lPRXhXdFF2NjRyaHIwX3V0cG8zVFk5cHFNQ1JZRGtlU2RnMjBXbWV3ZDNMWjZ0WDlPOC1mZk1iM0QyYXBFZXViZmc1djJfeFd0OWF4OUlvRkV2dXpTSWpqRkJ2RlNlSGNpdzZFTUliZldIYmQ2Z3NER2hDUm1FRjBRaDI3T3VfSlBUNFNvMHFVREEwd2lpd0xV?oc=5</t>
         </is>
       </c>
     </row>
@@ -1142,31 +1142,31 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Liverpool sign Víctor Muñoz for £34.5m in first arrival of Andoni Iraola era</t>
+          <t>World Cup: Florian Wirtz features as Germany book place in last 32 - Liverpool FC</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The Guardian</t>
+          <t>Liverpool FC</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G21" t="n">
-        <v>76.5</v>
+        <v>77</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.theguardian.com/football/2026/jun/18/victor-munoz-liverpool-newcastle-andoni-iraola-transfer-news</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNeVdTY0dsS0dqeEcwaWMycnhXNWo5M0RscDRuT194ckdxUUxEeEJma2swSFdTQUFkSXNzNllGNTVLRWt2QkFtbTlzQkZTWmxoVWpseXZsdnJXdkY3UTVtbThGNXZxVDVMSGduRHpkWnh4REl1NWd0Q3dPcnpES1U2OHR6OTVaWEJ3bHdOUlNaYXhtY3Z0ZWlr0gGfAUFVX3lxTE82aVdzMi1EbFg5RnFrbGV2bmxIVlZjOTZnekJ5bmZLOTFWazZIZzZpb2hyYllDZmdISDJwZVIzVFEyTlRwcWpTTGUwa2swZzByMmtRc0U2dHlRemV6RG5tbkxfMU5oQk1mZWZHTmUyNE5VanNYR0p1LXQ5NmxhTWxWT3kxQ1NUTkEyX3c5Wll2OEotNDlqaUVHbkVUdEVSaw?oc=5</t>
         </is>
       </c>
     </row>
@@ -1176,31 +1176,31 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Transfer rumors, news: Tottenham eye move for Liverpool's Gakpo - ESPN</t>
+          <t>Cody Gakpo Tottenham Interest Confirmed As Liverpool Delay Transfer Decision - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ESPN</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F22" t="n">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G22" t="n">
-        <v>75.7</v>
+        <v>77</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPYlo1NGNQeEp5U3hDME1uU0JHN050VjhUZTFPSk1lVk85QjVha2JvY3BqdGo5NE5IU0RaMUE0NTlJbERqaGRPQV9TakQ0UkplQlUzMEdHb01kTjRwVWt2cGotaEdWeWVvSXVzR2YtY3dpZE51SnRObDN4NGFrYmFTZGNjNmNHcm1WQ1l5cDUtTHR0WC1Bd1R2WDM5LXR3YS1QY19BaTBn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimAFBVV95cUxNRmhFRk90ajR2WmowQUt1SUZGR3BaaXl0d2dmWW1aODV1NzhtakVfdVdYb01RcXZuZUg5T1ljdnhyR0VqeE9QSnkybmVNN1ZBWjlvc2piWWNSWWVRSzVmTVRmdkJTcG9XWmlINzRPNTU1MEhoR1czaC1yUGNjTmliSlkxZHY3OEpBeHljZHNacHhpWjBESkZFXw?oc=5</t>
         </is>
       </c>
     </row>
@@ -1210,31 +1210,31 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Fabrizio Romano reveals whether Liverpool will sell Cody Gakpo to Tottenham - Football365</t>
+          <t>Liverpool sign Víctor Muñoz for £34.5m in first arrival of Andoni Iraola era</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Football365</t>
+          <t>The Guardian</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>9</v>
       </c>
       <c r="F23" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G23" t="n">
-        <v>75.59999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX2J6X01KNm0yYVFHWHNSMmdNRTc0Yk9zaVpyTmIycjByVGIxOXYxSy12Q0xEZWU1dHY1cVYyUjB4cTZRd2pwMVcwU2JoV1l1OWNjd0xDalhqbDYzb1lybVA5Qmc3UUNTcmpuN1QwbFNOLWJ1c0JqS1RkU2pZbWU1MHZhc3hOV0VBSUpjdEdkaHdYdGE3bGFYZmJR?oc=5</t>
+          <t>https://www.theguardian.com/football/2026/jun/18/victor-munoz-liverpool-newcastle-andoni-iraola-transfer-news</t>
         </is>
       </c>
     </row>
@@ -1244,31 +1244,31 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Superb £86m Liverpool swoop boosted by Fabrizio Romano as rival deal collapses - MSN</t>
+          <t>Liverpool Transfer News: Victor Muñoz signs six-year deal after US medical - readliverpoolfc.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>readliverpoolfc.com</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F24" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G24" t="n">
-        <v>75.59999999999999</v>
+        <v>76</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOV2JMc09SY1dLRC01Uks2UW84ZHNlQThGSFp0d3FLZ190SGQ3TWRMUzNHcEdGYnBQYmFtNjgwWkw4SWozN3dfZmVuRHQ1RnVxZVNkRXpvX0xHZUdXLWpHWHlSQW1yeHNKc2VKSkNBc3g0Y2pDZXlwcHNQNWE1LXBLb1FjZWhSSlFoaWQ1QlhWWHdZd21BYVV3SUF5N2JPZ2lJdlhleHBJNW9BM2t3eGU4WHJOSV9SWUROSTRSWXZwQzBaRGxLWUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNUGNKZjhPRzZaU3ZiQWpCZF9YTzViRHVTYjlpTDZEWjkzTVZidHRlUjhoNWg5bmNHYjI3Tkp1cHJqSjdZR244YzVpZlYtODhxZ2hFR3lwUC1JZTVKUzhZVjZNSWV0MUpxV3pUcXUwYzhpWDV5cmI2YmlFV3oxNUVLNDh3?oc=5</t>
         </is>
       </c>
     </row>
@@ -1278,31 +1278,31 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Liverpool rocked as Arsenal 'pushing' to complete £60m signing 'now' – Fabrizio Romano - MSN</t>
+          <t>Transfer rumors, news: Tottenham eye move for Liverpool's Gakpo - ESPN</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>ESPN</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="G25" t="n">
-        <v>75.59999999999999</v>
+        <v>75.7</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiowNBVV95cUxPcEZOa0hxYnNKMmVhUVk5UzYwSWtMcmJidjRibGJueHJubXhuVUs3WVZpR2NfVmZ2b0FJZU0tbmxGYzZlc3ZvSk81RWdnYU1nQ2VyM0ctbm1UOVhrRmp3SlBucVIwMEk5QklMcEFFdEZaYWRWaVdDRHZqLWJXb2t6MHVrdFJYamJpbjhWYnVnX0taYmJOZVpPNmZySlJKZEc2OWRLU0FJc2ZtWU9zd3FFdnB3VUN6b1lVeG9ZYlh1U2lDdGxwUEw5TTVHUVMwVVpFX05VZ0JSbUN1X01lSjE1d3hMR2dvemZlZ25wQXJEd0l2R081SUVfRndKSjlHajRaZUZTMG00RXloemIyT015ak5DN2lxY0pJSVhqeXV6UHBxeE9pa1NweTB0OXg3eXJ3MUdwZDZ3cVk2MnpCNC13ZmJ4cEhIWnB4cnJrVGFnTDR3NHhqZUk0T3BIMlNHRFlXMHY0OG9hbmNVTnhqVGUtS2RmOXlEVlByQWhnajNnQ1lWZVA5V2dDd2tBWDY2aGdOY2hkODBaUkUxaVBqZERvMVhNWQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxPYlo1NGNQeEp5U3hDME1uU0JHN050VjhUZTFPSk1lVk85QjVha2JvY3BqdGo5NE5IU0RaMUE0NTlJbERqaGRPQV9TakQ0UkplQlUzMEdHb01kTjRwVWt2cGotaEdWeWVvSXVzR2YtY3dpZE51SnRObDN4NGFrYmFTZGNjNmNHcm1WQ1l5cDUtTHR0WC1Bd1R2WDM5LXR3YS1QY19BaTBn?oc=5</t>
         </is>
       </c>
     </row>
@@ -1312,17 +1312,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fabrizio Romano claims Liverpool could sell £55m midfielder after Andoni Iraola arrival – good proposal - MSN</t>
+          <t>Fabrizio Romano reveals whether Liverpool will sell Cody Gakpo to Tottenham - Football365</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MSN</t>
+          <t>Football365</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMimANBVV95cUxPUUgxYkNpOFpmNmpBUlhyV0lFZG5PbE5sMG9sYXNFUE9aM2lMVy0tQ0RYaGQ0ZDJ3Vzhoc2IwN0dCSXhiTUlDZjVsaDFJNTF2Q1RfUkljSWh6VlFTbl9VSWFNXzNsckl5VlE4cFEyODh1Zm1qWXJ3MWF3cF9fWjdndkhLOTVsTTF6NURuU042T0d4bkdvbjZhTzBaN0VfMzhMaEdLaXFuM0x0WjdMSlVIYVd2RlNIVUNYeWx0WlZqRDQyUUxWVnpBR3NzdzNBa3lIdGVvSEpMN0U1SmtYdU1HWWRYbEtlYXRJaDhFZFZnMTZmSHpjZFE2RnZDemhKakFrczRBYjYzaTZweW9SRDJyd2VNdFNVNTM0X2J2dEpTa1NLZ052X3FHR2h6YWJFQnRCQ0xMVWV0cGxPUFFHWWNHUnFqV19BS0R4eHpMeUhzQXdobDFNUC1Db2JySkV4ZVBDOFNKT0VWNHNGQkdEbVlqeVc2WksxRVdHSFJtSTFETjRiOUVaUUZLQzdZTk1tTkVlUk8xNHNXaHM?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOX2J6X01KNm0yYVFHWHNSMmdNRTc0Yk9zaVpyTmIycjByVGIxOXYxSy12Q0xEZWU1dHY1cVYyUjB4cTZRd2pwMVcwU2JoV1l1OWNjd0xDalhqbDYzb1lybVA5Qmc3UUNTcmpuN1QwbFNOLWJ1c0JqS1RkU2pZbWU1MHZhc3hOV0VBSUpjdEdkaHdYdGE3bGFYZmJR?oc=5</t>
         </is>
       </c>
     </row>
@@ -1346,17 +1346,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fabrizio Romano confirms Liverpool missed out on perfect Conor Bradley replacement - Anfield Watch</t>
+          <t>Superb £86m Liverpool swoop boosted by Fabrizio Romano as rival deal collapses - MSN</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Anfield Watch</t>
+          <t>MSN</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOVWtUSjlBeHRjaHh0QmREMHpEU05EaEhQZnpwNVFqRGkyWVdNVUpCUE5tNEJKcFoyRzhhMUtFZE5NSkp6MG5aY0ZzaVVPMWpkRHNjbmFEckFRUENYZGViSno5ckxTbmVMcGFiSE14N1ZwcTBFVUpJLXI4VjV5Z2tRVnZBTklja1ZsaGVBbGxSNFdwdzMtQzEzazBMTDMxZlJwTVZiclZSVHV0UUszUHNFbVI2MGJ2eWVwU19CVEdGN3Bqa1ZQWXpIaUhkak4?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxOV2JMc09SY1dLRC01Uks2UW84ZHNlQThGSFp0d3FLZ190SGQ3TWRMUzNHcEdGYnBQYmFtNjgwWkw4SWozN3dfZmVuRHQ1RnVxZVNkRXpvX0xHZUdXLWpHWHlSQW1yeHNKc2VKSkNBc3g0Y2pDZXlwcHNQNWE1LXBLb1FjZWhSSlFoaWQ1QlhWWHdZd21BYVV3SUF5N2JPZ2lJdlhleHBJNW9BM2t3eGU4WHJOSV9SWUROSTRSWXZwQzBaRGxLWUE?oc=5</t>
         </is>
       </c>
     </row>
@@ -1385,12 +1385,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fabrizio Romano confirms Liverpool talks for sensational midfielder - Anfield Watch</t>
+          <t>Liverpool rocked as Arsenal 'pushing' to complete £60m signing 'now' – Fabrizio Romano - MSN</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Anfield Watch</t>
+          <t>MSN</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPdVRCMW5CSVlJc2pwei1ZY044dVktUzczWEdpbUVNcm8yU0FpWU9lUTJIUkdTX29BSUYzY1hkeFJGaHF2R0x5NHI1b0RDWTF2WkttUk8xdkVWWTdCVl9PZm9tVEZJcmFraTRBaDc2Y0tXS1pwUUlZa0pYQl9wU2dWbDFKdjE3TExPVkVNaFFkSXUyNmhIT3loY1pDNDlESFRMMzliX1BDckJGanpUUWFuM0QxUHRDSVNz?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilAJBVV95cUxQUllDeU53RGFUSm9DTTA1XzhjMVZGQ0UyMW5SUnM2RlFtaENEc0FfSTZZT3JGQXFtM0lhR2NMdTdNOTdBYW5iYlJNeGxqd1dUdDR2bk9ySW5lLTMxMUg1b29pVms0OXljZGhZSjEwWlZvd24yZDFrcUZVY2Z3THlqWnJLakdidnI0SnZzSE11YzRZaWZfZlhNaVRiSnVkZnZRN0E1eGl4c2RwaFpSZTVsZWNiWURtRUlmQ09KVkVaVlozam1USm51akRacUlsaGJvWmZWMmpuRkxENExWY05YODQtR0ZEV1U1UXZ6Q0hIdnJqTC1nNHN3RXNsUlVSaDFqM2ZDR243X0pLczJobksyanlINHg?oc=5</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ornstein Drops €100M BOMBA! Liverpool’s Diomande Move REJECTED Jake Gyllenhaal (jKheLn24tz) - Fathom Journal</t>
+          <t>Fabrizio Romano confirms Liverpool missed out on perfect Conor Bradley replacement - Anfield Watch</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Fathom Journal</t>
+          <t>Anfield Watch</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1qQXI1OWcyNmNaeW5GekhZUlBCTGNHVU1nQnZZbWctV1BUNnlGdHRmdU9CNFlHa3JWNEpGb2tUNmo4ZGtIVkJ4RURkLXZqNjBPX1ZWd3h3T0RHMHF2c2pacnhIYmw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMizAFBVV95cUxOVWtUSjlBeHRjaHh0QmREMHpEU05EaEhQZnpwNVFqRGkyWVdNVUpCUE5tNEJKcFoyRzhhMUtFZE5NSkp6MG5aY0ZzaVVPMWpkRHNjbmFEckFRUENYZGViSno5ckxTbmVMcGFiSE14N1ZwcTBFVUpJLXI4VjV5Z2tRVnZBTklja1ZsaGVBbGxSNFdwdzMtQzEzazBMTDMxZlJwTVZiclZSVHV0UUszUHNFbVI2MGJ2eWVwU19CVEdGN3Bqa1ZQWXpIaUhkak4?oc=5</t>
         </is>
       </c>
     </row>
@@ -1453,26 +1453,26 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Liverpool transfer news LIVE: Yan Diomande deal, Bradley Barcola boost, Eduardo Camavinga contact</t>
+          <t>Fabrizio Romano confirms Liverpool talks for sensational midfielder - Anfield Watch</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Liverpool Echo</t>
+          <t>Anfield Watch</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F30" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G30" t="n">
-        <v>75.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.liverpoolecho.co.uk/sport/football/football-news/liverpool-transfer-latest-34162535</t>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPdVRCMW5CSVlJc2pwei1ZY044dVktUzczWEdpbUVNcm8yU0FpWU9lUTJIUkdTX29BSUYzY1hkeFJGaHF2R0x5NHI1b0RDWTF2WkttUk8xdkVWWTdCVl9PZm9tVEZJcmFraTRBaDc2Y0tXS1pwUUlZa0pYQl9wU2dWbDFKdjE3TExPVkVNaFFkSXUyNmhIT3loY1pDNDlESFRMMzliX1BDckJGanpUUWFuM0QxUHRDSVNz?oc=5</t>
         </is>
       </c>
     </row>
@@ -1482,31 +1482,31 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Liverpool transfer latest: Bradley Barcola boost as Yan Diomande agreement reached</t>
+          <t>Ornstein Drops €100M BOMBA! Liverpool’s Diomande Move REJECTED Jake Gyllenhaal (jKheLn24tz) - Fathom Journal</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Liverpool Echo</t>
+          <t>Fathom Journal</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F31" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="G31" t="n">
-        <v>75.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.liverpoolecho.co.uk/sport/football/football-news/liverpool-barcola-diomande-summer-transfers-34172877</t>
+          <t>https://news.google.com/rss/articles/CBMiZEFVX3lxTE1qQXI1OWcyNmNaeW5GekhZUlBCTGNHVU1nQnZZbWctV1BUNnlGdHRmdU9CNFlHa3JWNEpGb2tUNmo4ZGtIVkJ4RURkLXZqNjBPX1ZWd3h3T0RHMHF2c2pacnhIYmw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>